<commit_message>
Correct STU002 node reach normalization
</commit_message>
<xml_diff>
--- a/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_simplified_flop_strategy.xlsx
+++ b/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_simplified_flop_strategy.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R898a57b99001444d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="R5b3130a631b247c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="R7d5abbb4e38d4af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="R38d0c231ecb84453"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R321b1f94e2c642ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="R193ea15022ab4230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="Rab7e4231b17e43ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loss audit" sheetId="8" r:id="R838eed46b5c84335"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="9" r:id="R26143e3b3cd24f75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0762da437f1142a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="Reb74083291e24c08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="R388ae352947441e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="Rd4ed38081c3f44e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R56a0716b901c4948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="R382f82c3baf14cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="R85b720df3d294012"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loss audit" sheetId="8" r:id="R2c763d4dc89f48b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="9" r:id="Rdcf555da0df04f20"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -914,7 +914,7 @@
         <x:v>80553</x:v>
       </x:c>
       <x:c r="E7" s="21" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9362318512399077</x:v>
       </x:c>
       <x:c r="F7" s="19" t="str">
         <x:v>check 44.1%; bet 55.9%</x:v>
@@ -926,7 +926,7 @@
         <x:v>0.0014611368670458358</x:v>
       </x:c>
       <x:c r="I7" s="22" t="n">
-        <x:v>0.0014611368670458358</x:v>
+        <x:v>0.0013679628739492018</x:v>
       </x:c>
       <x:c r="J7" s="27" t="n">
         <x:v>377</x:v>
@@ -978,7 +978,7 @@
         <x:v>75236</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
-        <x:v>0.0727232809275815</x:v>
+        <x:v>0.0680858519310695</x:v>
       </x:c>
       <x:c r="F9" s="19" t="str">
         <x:v>fold 39.2%; call 60.8%</x:v>
@@ -990,7 +990,7 @@
         <x:v>0.01944839218345448</x:v>
       </x:c>
       <x:c r="I9" s="22" t="n">
-        <x:v>0.0014143508883471402</x:v>
+        <x:v>0.001324160350500051</x:v>
       </x:c>
       <x:c r="J9" s="27" t="n">
         <x:v>373</x:v>
@@ -1010,7 +1010,7 @@
         <x:v>80553</x:v>
       </x:c>
       <x:c r="E10" s="21" t="n">
-        <x:v>0.06811148703379341</x:v>
+        <x:v>0.06376814359635138</x:v>
       </x:c>
       <x:c r="F10" s="19" t="str">
         <x:v>fold 28.0%; call 59.0%; raise 12.9%</x:v>
@@ -1022,7 +1022,7 @@
         <x:v>0.013529385518906738</x:v>
       </x:c>
       <x:c r="I10" s="22" t="n">
-        <x:v>0.0009215065663462088</x:v>
+        <x:v>0.0008627437985400419</x:v>
       </x:c>
       <x:c r="J10" s="27" t="n">
         <x:v>377</x:v>

</xml_diff>

<commit_message>
Simplify draw classes and add full UTG BTN study
</commit_message>
<xml_diff>
--- a/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_simplified_flop_strategy.xlsx
+++ b/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_simplified_flop_strategy.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb13343f659b24752"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="R3f0608df1cb44807"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="Ra0c82b68229748c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="R11a1db8205c74383"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R5ad1bcf939f84d09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="R2396ec983cb14ee3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="Rb082b799ce024de9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="8" r:id="R762a3062d6d94486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R69ec1f52de3345c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="Rd5c42a3f64dc40f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="R780dc711b1514677"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="Rde145329db484f57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R4dc32074d93e4a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="R4364952ff6c5439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="R5e0981b401044771"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="8" r:id="Re844cf4617ea4045"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -307,7 +307,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="92">
+  <x:cellXfs count="91">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -506,9 +506,6 @@
     <x:xf numFmtId="0" fontId="11" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
@@ -545,9 +542,6 @@
     <x:xf numFmtId="0" fontId="11" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
@@ -555,6 +549,9 @@
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -820,7 +817,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="7" t="str">
-        <x:v>13 категорий рук × 13 узких категорий флопов B13. Чистое действие или строгий микс 50/50.</x:v>
+        <x:v>11 категорий рук × 13 узких категорий флопов B13. Чистое действие или строгий микс 50/50.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -867,7 +864,7 @@
         <x:v>Loss от root, bb</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
-        <x:v>Добавка к 13×B13, bb</x:v>
+        <x:v>Добавка к B13, bb</x:v>
       </x:c>
       <x:c r="I5" s="12" t="str">
         <x:v>Комбо reach &gt; 0</x:v>
@@ -893,10 +890,10 @@
         <x:v>X 97.2%; D 2.8%</x:v>
       </x:c>
       <x:c r="F6" s="17" t="n">
-        <x:v>0.00021348805069739733</x:v>
+        <x:v>0.00021120267391907833</x:v>
       </x:c>
       <x:c r="G6" s="17" t="n">
-        <x:v>0.00021348805069738782</x:v>
+        <x:v>0.0002112026739190689</x:v>
       </x:c>
       <x:c r="H6" s="17" t="n">
         <x:v>0</x:v>
@@ -905,7 +902,7 @@
         <x:v>106381</x:v>
       </x:c>
       <x:c r="J6" s="18" t="n">
-        <x:v>126</x:v>
+        <x:v>119</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -922,13 +919,13 @@
         <x:v>X 44.1%; B 55.9%</x:v>
       </x:c>
       <x:c r="E7" s="15" t="str">
-        <x:v>X 38.2%; B 61.8%</x:v>
+        <x:v>X 38.7%; B 61.3%</x:v>
       </x:c>
       <x:c r="F7" s="17" t="n">
-        <x:v>0.0022099723261542375</x:v>
+        <x:v>0.0020744965595297935</x:v>
       </x:c>
       <x:c r="G7" s="17" t="n">
-        <x:v>0.0020690464821042547</x:v>
+        <x:v>0.0019422097543193115</x:v>
       </x:c>
       <x:c r="H7" s="17" t="n">
         <x:v>0</x:v>
@@ -937,7 +934,7 @@
         <x:v>80553</x:v>
       </x:c>
       <x:c r="J7" s="18" t="n">
-        <x:v>135</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -954,13 +951,13 @@
         <x:v>F 47.9%; C 39.1%; R 13.0%</x:v>
       </x:c>
       <x:c r="E8" s="15" t="str">
-        <x:v>F 47.5%; C 40.8%; R 11.7%</x:v>
+        <x:v>F 51.8%; C 37.7%; R 10.5%</x:v>
       </x:c>
       <x:c r="F8" s="17" t="n">
-        <x:v>0.016859085175564843</x:v>
+        <x:v>0.019275265265655282</x:v>
       </x:c>
       <x:c r="G8" s="17" t="n">
-        <x:v>0.008824541885092161</x:v>
+        <x:v>0.010089241730006164</x:v>
       </x:c>
       <x:c r="H8" s="17" t="n">
         <x:v>0</x:v>
@@ -969,7 +966,7 @@
         <x:v>106308</x:v>
       </x:c>
       <x:c r="J8" s="18" t="n">
-        <x:v>126</x:v>
+        <x:v>119</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -986,13 +983,13 @@
         <x:v>F 39.2%; C 60.8%</x:v>
       </x:c>
       <x:c r="E9" s="15" t="str">
-        <x:v>F 39.0%; C 61.0%</x:v>
+        <x:v>F 40.7%; C 59.3%</x:v>
       </x:c>
       <x:c r="F9" s="17" t="n">
-        <x:v>0.03489997299599592</x:v>
+        <x:v>0.03349741908962209</x:v>
       </x:c>
       <x:c r="G9" s="17" t="n">
-        <x:v>0.0023761943938035964</x:v>
+        <x:v>0.002280700316208889</x:v>
       </x:c>
       <x:c r="H9" s="17" t="n">
         <x:v>0</x:v>
@@ -1001,7 +998,7 @@
         <x:v>75236</x:v>
       </x:c>
       <x:c r="J9" s="18" t="n">
-        <x:v>135</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1018,13 +1015,13 @@
         <x:v>F 28.0%; C 59.0%; R 12.9%</x:v>
       </x:c>
       <x:c r="E10" s="15" t="str">
-        <x:v>F 35.7%; C 58.3%; R 6.0%</x:v>
+        <x:v>F 35.5%; C 58.5%; R 6.0%</x:v>
       </x:c>
       <x:c r="F10" s="17" t="n">
-        <x:v>0.01628671477594084</x:v>
+        <x:v>0.015901470575785587</x:v>
       </x:c>
       <x:c r="G10" s="17" t="n">
-        <x:v>0.0010385735665449669</x:v>
+        <x:v>0.0010140072590698063</x:v>
       </x:c>
       <x:c r="H10" s="17" t="n">
         <x:v>0</x:v>
@@ -1033,7 +1030,7 @@
         <x:v>80553</x:v>
       </x:c>
       <x:c r="J10" s="18" t="n">
-        <x:v>135</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1050,13 +1047,13 @@
         <x:v>F 41.5%; C 58.5%</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
-        <x:v>F 32.3%; C 67.7%</x:v>
+        <x:v>F 34.2%; C 65.8%</x:v>
       </x:c>
       <x:c r="F11" s="17" t="n">
-        <x:v>0.13549392861734005</x:v>
+        <x:v>0.06407484830732571</x:v>
       </x:c>
       <x:c r="G11" s="17" t="n">
-        <x:v>0.0011170914017892806</x:v>
+        <x:v>0.0005282706232337096</x:v>
       </x:c>
       <x:c r="H11" s="17" t="n">
         <x:v>0</x:v>
@@ -1065,7 +1062,7 @@
         <x:v>57240</x:v>
       </x:c>
       <x:c r="J11" s="18" t="n">
-        <x:v>120</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1155,7 +1152,7 @@
       <x:c r="D16" s="23"/>
       <x:c r="E16" s="3"/>
       <x:c r="F16" s="24" t="str">
-        <x:v>13 категорий рук и правила BDFD/Gutshot/OESD одинаковы в обеих таблицах.</x:v>
+        <x:v>11 категорий рук: 7 made, OESD, Gutshot, 2 overcards + BDFD и Air.</x:v>
       </x:c>
       <x:c r="G16" s="24"/>
       <x:c r="H16" s="24"/>
@@ -1544,46 +1541,46 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="37" t="str">
         <x:v>Top pair</x:v>
       </x:c>
-      <x:c r="B9" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="C9" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="D9" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E9" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F9" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G9" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H9" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I9" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="J9" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="K9" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="L9" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="M9" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="N9" s="61" t="str">
+      <x:c r="B9" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C9" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D9" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E9" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F9" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G9" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H9" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I9" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="J9" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="K9" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="L9" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="M9" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="N9" s="60" t="str">
         <x:v>X/D</x:v>
       </x:c>
     </x:row>
@@ -1765,31 +1762,31 @@
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="37" t="str">
-        <x:v>2 overcards</x:v>
-      </x:c>
-      <x:c r="B14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D14" s="49" t="str">
-        <x:v>—</x:v>
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B14" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C14" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D14" s="41" t="str">
+        <x:v>X</x:v>
       </x:c>
       <x:c r="E14" s="57" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="F14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I14" s="57" t="str">
-        <x:v>—</x:v>
+      <x:c r="F14" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G14" s="60" t="str">
+        <x:v>X/D</x:v>
+      </x:c>
+      <x:c r="H14" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I14" s="56" t="str">
+        <x:v>X</x:v>
       </x:c>
       <x:c r="J14" s="41" t="str">
         <x:v>X</x:v>
@@ -1803,43 +1800,43 @@
       <x:c r="M14" s="56" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="N14" s="56" t="str">
-        <x:v>X</x:v>
+      <x:c r="N14" s="60" t="str">
+        <x:v>X/D</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="50" t="str">
-        <x:v>2 overcards + draw</x:v>
-      </x:c>
-      <x:c r="B15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H15" s="53" t="str">
-        <x:v>—</x:v>
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B15" s="51" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C15" s="58" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D15" s="51" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E15" s="58" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F15" s="51" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G15" s="58" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H15" s="51" t="str">
+        <x:v>X</x:v>
       </x:c>
       <x:c r="I15" s="58" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="J15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="K15" s="59" t="str">
-        <x:v>—</x:v>
+      <x:c r="J15" s="51" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="K15" s="58" t="str">
+        <x:v>X</x:v>
       </x:c>
       <x:c r="L15" s="58" t="str">
         <x:v>X</x:v>
@@ -1852,179 +1849,91 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="37" t="str">
-        <x:v>A-high</x:v>
-      </x:c>
-      <x:c r="B16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I16" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="J16" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="K16" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="L16" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="M16" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="N16" s="60" t="str">
+      <x:c r="A16" s="50" t="str">
+        <x:v>2 overcards + BDFD</x:v>
+      </x:c>
+      <x:c r="B16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="L16" s="58" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="M16" s="58" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="N16" s="61" t="str">
         <x:v>X/D</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="50" t="str">
-        <x:v>A-high + draw</x:v>
-      </x:c>
-      <x:c r="B17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H17" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I17" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="J17" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="K17" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="L17" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="M17" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="N17" s="61" t="str">
-        <x:v>X/D</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="37" t="str">
+      <x:c r="A17" s="37" t="str">
         <x:v>Air</x:v>
       </x:c>
-      <x:c r="B18" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="C18" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="D18" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E18" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F18" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G18" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H18" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I18" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="J18" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="K18" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="L18" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="M18" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="N18" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="37" t="str">
-        <x:v>Air + draw</x:v>
-      </x:c>
-      <x:c r="B19" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="C19" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="D19" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E19" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F19" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G19" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H19" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I19" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="J19" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="K19" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="L19" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="M19" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="N19" s="60" t="str">
-        <x:v>X/D</x:v>
+      <x:c r="B17" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C17" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D17" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E17" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F17" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G17" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H17" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I17" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="J17" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="K17" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="L17" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="M17" s="56" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="N17" s="56" t="str">
+        <x:v>X</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2217,40 +2126,40 @@
       <x:c r="B7" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C7" s="70" t="str">
+      <x:c r="C7" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="D7" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="E7" s="70" t="str">
+      <x:c r="E7" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="F7" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G7" s="70" t="str">
+      <x:c r="G7" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H7" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="I7" s="70" t="str">
+      <x:c r="I7" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="J7" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="K7" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="L7" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="M7" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="N7" s="70" t="str">
+      <x:c r="K7" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="L7" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="M7" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="N7" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
@@ -2279,19 +2188,19 @@
       <x:c r="H8" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="I8" s="70" t="str">
+      <x:c r="I8" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="J8" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="K8" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="L8" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="M8" s="70" t="str">
+      <x:c r="K8" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="L8" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="M8" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="N8" s="60" t="str">
@@ -2299,46 +2208,46 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="37" t="str">
         <x:v>Top pair</x:v>
       </x:c>
-      <x:c r="B9" s="66" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="C9" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="D9" s="67" t="str">
+      <x:c r="B9" s="65" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="C9" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="E9" s="61" t="str">
+      <x:c r="E9" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="F9" s="67" t="str">
+      <x:c r="F9" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="G9" s="61" t="str">
+      <x:c r="G9" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="H9" s="66" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="I9" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="J9" s="67" t="str">
+      <x:c r="H9" s="65" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="I9" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J9" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="K9" s="61" t="str">
+      <x:c r="K9" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="L9" s="61" t="str">
+      <x:c r="L9" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="M9" s="61" t="str">
+      <x:c r="M9" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="N9" s="71" t="str">
+      <x:c r="N9" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
@@ -2382,7 +2291,7 @@
       <x:c r="M10" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="N10" s="70" t="str">
+      <x:c r="N10" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
@@ -2405,7 +2314,7 @@
       <x:c r="F11" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G11" s="70" t="str">
+      <x:c r="G11" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H11" s="45" t="str">
@@ -2417,7 +2326,7 @@
       <x:c r="J11" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="K11" s="70" t="str">
+      <x:c r="K11" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="L11" s="60" t="str">
@@ -2426,7 +2335,7 @@
       <x:c r="M11" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="N11" s="70" t="str">
+      <x:c r="N11" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
@@ -2437,25 +2346,25 @@
       <x:c r="B12" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C12" s="70" t="str">
+      <x:c r="C12" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="D12" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="E12" s="70" t="str">
+      <x:c r="E12" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="F12" s="65" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G12" s="70" t="str">
+      <x:c r="G12" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H12" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="I12" s="70" t="str">
+      <x:c r="I12" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="J12" s="45" t="str">
@@ -2493,7 +2402,7 @@
       <x:c r="F13" s="67" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="G13" s="71" t="str">
+      <x:c r="G13" s="70" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="H13" s="66" t="str">
@@ -2520,266 +2429,178 @@
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="37" t="str">
-        <x:v>2 overcards</x:v>
-      </x:c>
-      <x:c r="B14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D14" s="49" t="str">
-        <x:v>—</x:v>
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B14" s="65" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="C14" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D14" s="65" t="str">
+        <x:v>B</x:v>
       </x:c>
       <x:c r="E14" s="57" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="F14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="J14" s="45" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="K14" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="L14" s="60" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="M14" s="60" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="N14" s="60" t="str">
-        <x:v>X/B</x:v>
+      <x:c r="F14" s="65" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G14" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H14" s="65" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="I14" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J14" s="65" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K14" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="L14" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="M14" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="N14" s="69" t="str">
+        <x:v>B</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="50" t="str">
-        <x:v>2 overcards + draw</x:v>
-      </x:c>
-      <x:c r="B15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I15" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="J15" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="K15" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="L15" s="61" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="M15" s="61" t="str">
-        <x:v>X/B</x:v>
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B15" s="66" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="C15" s="70" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D15" s="66" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E15" s="70" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F15" s="66" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G15" s="70" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H15" s="66" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="I15" s="70" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J15" s="66" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K15" s="70" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="L15" s="70" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="M15" s="70" t="str">
+        <x:v>B</x:v>
       </x:c>
       <x:c r="N15" s="61" t="str">
         <x:v>X/B</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="37" t="str">
-        <x:v>A-high</x:v>
-      </x:c>
-      <x:c r="B16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I16" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="J16" s="45" t="str">
+      <x:c r="A16" s="50" t="str">
+        <x:v>2 overcards + BDFD</x:v>
+      </x:c>
+      <x:c r="B16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J16" s="51" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="K16" s="58" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="L16" s="61" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="K16" s="60" t="str">
+      <x:c r="M16" s="58" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="N16" s="61" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="L16" s="60" t="str">
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="37" t="str">
+        <x:v>Air</x:v>
+      </x:c>
+      <x:c r="B17" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="M16" s="60" t="str">
+      <x:c r="C17" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="N16" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="50" t="str">
-        <x:v>A-high + draw</x:v>
-      </x:c>
-      <x:c r="B17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H17" s="66" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="I17" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="J17" s="66" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="K17" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="L17" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="M17" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="N17" s="61" t="str">
+      <x:c r="D17" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="37" t="str">
-        <x:v>Air</x:v>
-      </x:c>
-      <x:c r="B18" s="45" t="str">
+      <x:c r="E17" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="C18" s="60" t="str">
+      <x:c r="F17" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="D18" s="45" t="str">
+      <x:c r="G17" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="E18" s="60" t="str">
+      <x:c r="H17" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="F18" s="45" t="str">
+      <x:c r="I17" s="69" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J17" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="G18" s="60" t="str">
+      <x:c r="K17" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="H18" s="45" t="str">
+      <x:c r="L17" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="I18" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="J18" s="65" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="K18" s="60" t="str">
+      <x:c r="M17" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="L18" s="60" t="str">
+      <x:c r="N17" s="60" t="str">
         <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="M18" s="60" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="N18" s="60" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="37" t="str">
-        <x:v>Air + draw</x:v>
-      </x:c>
-      <x:c r="B19" s="65" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="C19" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="D19" s="65" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="E19" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="F19" s="65" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G19" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="H19" s="65" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="I19" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="J19" s="65" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="K19" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="L19" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="M19" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="N19" s="70" t="str">
-        <x:v>B</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2972,40 +2793,40 @@
       <x:c r="B7" s="45" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="C7" s="82" t="str">
+      <x:c r="C7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="D7" s="75" t="str">
+      <x:c r="D7" s="74" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="E7" s="82" t="str">
+      <x:c r="E7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="F7" s="75" t="str">
+      <x:c r="F7" s="74" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="G7" s="82" t="str">
+      <x:c r="G7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="H7" s="45" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="I7" s="82" t="str">
+      <x:c r="I7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="J7" s="75" t="str">
+      <x:c r="J7" s="74" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="K7" s="82" t="str">
+      <x:c r="K7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="L7" s="82" t="str">
+      <x:c r="L7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="M7" s="82" t="str">
+      <x:c r="M7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="N7" s="82" t="str">
+      <x:c r="N7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
     </x:row>
@@ -3054,46 +2875,46 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="37" t="str">
         <x:v>Top pair</x:v>
       </x:c>
-      <x:c r="B9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="C9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="D9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="N9" s="58" t="str">
+      <x:c r="B9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="L9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="N9" s="56" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3233,40 +3054,40 @@
       <x:c r="A13" s="50" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C13" s="83" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E13" s="83" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F13" s="80" t="str">
+      <x:c r="B13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C13" s="81" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E13" s="81" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F13" s="79" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="G13" s="61" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="H13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I13" s="83" t="str">
+      <x:c r="H13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I13" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="J13" s="67" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="K13" s="83" t="str">
+      <x:c r="K13" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="L13" s="61" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="M13" s="83" t="str">
+      <x:c r="M13" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="N13" s="58" t="str">
@@ -3275,81 +3096,81 @@
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="37" t="str">
-        <x:v>2 overcards</x:v>
-      </x:c>
-      <x:c r="B14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D14" s="49" t="str">
-        <x:v>—</x:v>
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="C14" s="60" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="D14" s="74" t="str">
+        <x:v>R</x:v>
       </x:c>
       <x:c r="E14" s="57" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="F14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="J14" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L14" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="M14" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="N14" s="84" t="str">
-        <x:v>F</x:v>
+      <x:c r="F14" s="74" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="G14" s="80" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="H14" s="45" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="I14" s="60" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="J14" s="74" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="K14" s="80" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="L14" s="80" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="M14" s="80" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="N14" s="80" t="str">
+        <x:v>R</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="50" t="str">
-        <x:v>2 overcards + draw</x:v>
-      </x:c>
-      <x:c r="B15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="K15" s="59" t="str">
-        <x:v>—</x:v>
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B15" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C15" s="61" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="D15" s="67" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="E15" s="61" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="F15" s="67" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="G15" s="61" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="H15" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I15" s="61" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="J15" s="67" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="K15" s="61" t="str">
+        <x:v>C/R</x:v>
       </x:c>
       <x:c r="L15" s="61" t="str">
         <x:v>C/R</x:v>
@@ -3362,179 +3183,91 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="37" t="str">
-        <x:v>A-high</x:v>
-      </x:c>
-      <x:c r="B16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="J16" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="M16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N16" s="60" t="str">
-        <x:v>F/R</x:v>
+      <x:c r="A16" s="50" t="str">
+        <x:v>2 overcards + BDFD</x:v>
+      </x:c>
+      <x:c r="B16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="L16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="N16" s="61" t="str">
+        <x:v>F/C</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="50" t="str">
-        <x:v>A-high + draw</x:v>
-      </x:c>
-      <x:c r="B17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H17" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J17" s="81" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="K17" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="L17" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="M17" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="N17" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="37" t="str">
+      <x:c r="A17" s="37" t="str">
         <x:v>Air</x:v>
       </x:c>
-      <x:c r="B18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="H18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="J18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="M18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="37" t="str">
-        <x:v>Air + draw</x:v>
-      </x:c>
-      <x:c r="B19" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="D19" s="45" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="E19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="F19" s="45" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="G19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="H19" s="45" t="str">
-        <x:v>F/R</x:v>
-      </x:c>
-      <x:c r="I19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="J19" s="45" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="K19" s="82" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="L19" s="82" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="M19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="N19" s="82" t="str">
-        <x:v>R</x:v>
+      <x:c r="B17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="J17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="K17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="L17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="M17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="N17" s="82" t="str">
+        <x:v>F</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3809,46 +3542,46 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="37" t="str">
         <x:v>Top pair</x:v>
       </x:c>
-      <x:c r="B9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="C9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="D9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="N9" s="58" t="str">
+      <x:c r="B9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="L9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="N9" s="56" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3903,7 +3636,7 @@
       <x:c r="B11" s="45" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="C11" s="84" t="str">
+      <x:c r="C11" s="82" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="D11" s="45" t="str">
@@ -3944,7 +3677,7 @@
       <x:c r="A12" s="37" t="str">
         <x:v>Third pair</x:v>
       </x:c>
-      <x:c r="B12" s="79" t="str">
+      <x:c r="B12" s="78" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="C12" s="56" t="str">
@@ -3988,16 +3721,16 @@
       <x:c r="A13" s="50" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C13" s="83" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E13" s="83" t="str">
+      <x:c r="B13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C13" s="81" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E13" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="F13" s="67" t="str">
@@ -4006,22 +3739,22 @@
       <x:c r="G13" s="58" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="H13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I13" s="83" t="str">
+      <x:c r="H13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I13" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="J13" s="67" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="K13" s="83" t="str">
+      <x:c r="K13" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="L13" s="61" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="M13" s="83" t="str">
+      <x:c r="M13" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="N13" s="58" t="str">
@@ -4030,75 +3763,75 @@
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="37" t="str">
-        <x:v>2 overcards</x:v>
-      </x:c>
-      <x:c r="B14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D14" s="49" t="str">
-        <x:v>—</x:v>
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B14" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D14" s="41" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="E14" s="57" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="F14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="J14" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K14" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L14" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="M14" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N14" s="84" t="str">
-        <x:v>F</x:v>
+      <x:c r="F14" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H14" s="45" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="I14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J14" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="L14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="N14" s="56" t="str">
+        <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="50" t="str">
-        <x:v>2 overcards + draw</x:v>
-      </x:c>
-      <x:c r="B15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I15" s="58" t="str">
-        <x:v>C</x:v>
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B15" s="67" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="C15" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D15" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E15" s="61" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="F15" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G15" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H15" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I15" s="61" t="str">
+        <x:v>F/C</x:v>
       </x:c>
       <x:c r="J15" s="51" t="str">
         <x:v>C</x:v>
@@ -4117,179 +3850,91 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="37" t="str">
-        <x:v>A-high</x:v>
-      </x:c>
-      <x:c r="B16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="J16" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="M16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N16" s="84" t="str">
-        <x:v>F</x:v>
+      <x:c r="A16" s="50" t="str">
+        <x:v>2 overcards + BDFD</x:v>
+      </x:c>
+      <x:c r="B16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J16" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="L16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="N16" s="58" t="str">
+        <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="50" t="str">
-        <x:v>A-high + draw</x:v>
-      </x:c>
-      <x:c r="B17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H17" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I17" s="61" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="J17" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="N17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="37" t="str">
+      <x:c r="A17" s="37" t="str">
         <x:v>Air</x:v>
       </x:c>
-      <x:c r="B18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="H18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="J18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L18" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="M18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N18" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="37" t="str">
-        <x:v>Air + draw</x:v>
-      </x:c>
-      <x:c r="B19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="C19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="D19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E19" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="F19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H19" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="N19" s="56" t="str">
-        <x:v>C</x:v>
+      <x:c r="B17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="J17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="K17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="L17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="M17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="N17" s="82" t="str">
+        <x:v>F</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4479,16 +4124,16 @@
       <x:c r="A7" s="37" t="str">
         <x:v>Two pair+</x:v>
       </x:c>
-      <x:c r="B7" s="75" t="str">
+      <x:c r="B7" s="74" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="C7" s="82" t="str">
+      <x:c r="C7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="D7" s="75" t="str">
+      <x:c r="D7" s="74" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="E7" s="82" t="str">
+      <x:c r="E7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="F7" s="45" t="str">
@@ -4500,22 +4145,22 @@
       <x:c r="H7" s="45" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="I7" s="82" t="str">
+      <x:c r="I7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="J7" s="75" t="str">
+      <x:c r="J7" s="74" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="K7" s="82" t="str">
+      <x:c r="K7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="L7" s="82" t="str">
+      <x:c r="L7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="M7" s="82" t="str">
+      <x:c r="M7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="N7" s="82" t="str">
+      <x:c r="N7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
     </x:row>
@@ -4541,7 +4186,7 @@
       <x:c r="G8" s="57" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="H8" s="75" t="str">
+      <x:c r="H8" s="74" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="I8" s="60" t="str">
@@ -4564,46 +4209,46 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="37" t="str">
         <x:v>Top pair</x:v>
       </x:c>
-      <x:c r="B9" s="67" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="C9" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="D9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H9" s="67" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="I9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="N9" s="58" t="str">
+      <x:c r="B9" s="45" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="C9" s="60" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="D9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="I9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="L9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="N9" s="56" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -4629,7 +4274,7 @@
       <x:c r="G10" s="56" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="H10" s="75" t="str">
+      <x:c r="H10" s="74" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="I10" s="60" t="str">
@@ -4702,13 +4347,13 @@
       <x:c r="B12" s="45" t="str">
         <x:v>F/R</x:v>
       </x:c>
-      <x:c r="C12" s="82" t="str">
+      <x:c r="C12" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="D12" s="45" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="E12" s="82" t="str">
+      <x:c r="E12" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="F12" s="45" t="str">
@@ -4743,13 +4388,13 @@
       <x:c r="A13" s="50" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="80" t="str">
+      <x:c r="B13" s="79" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="C13" s="61" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="D13" s="80" t="str">
+      <x:c r="D13" s="79" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="E13" s="61" t="str">
@@ -4761,7 +4406,7 @@
       <x:c r="G13" s="58" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="H13" s="80" t="str">
+      <x:c r="H13" s="79" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="I13" s="61" t="str">
@@ -4785,266 +4430,178 @@
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="37" t="str">
-        <x:v>2 overcards</x:v>
-      </x:c>
-      <x:c r="B14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D14" s="49" t="str">
-        <x:v>—</x:v>
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="C14" s="80" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="D14" s="45" t="str">
+        <x:v>C/R</x:v>
       </x:c>
       <x:c r="E14" s="57" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="F14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="J14" s="45" t="str">
-        <x:v>F/C</x:v>
+      <x:c r="F14" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H14" s="45" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="I14" s="60" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="J14" s="74" t="str">
+        <x:v>R</x:v>
       </x:c>
       <x:c r="K14" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="L14" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="M14" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N14" s="84" t="str">
-        <x:v>F</x:v>
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="L14" s="80" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="M14" s="80" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="N14" s="60" t="str">
+        <x:v>C/R</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="50" t="str">
-        <x:v>2 overcards + draw</x:v>
-      </x:c>
-      <x:c r="B15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H15" s="53" t="str">
-        <x:v>—</x:v>
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B15" s="67" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="C15" s="61" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="D15" s="67" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="E15" s="61" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="F15" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G15" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H15" s="67" t="str">
+        <x:v>F/R</x:v>
       </x:c>
       <x:c r="I15" s="61" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="J15" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K15" s="58" t="str">
-        <x:v>C</x:v>
+      <x:c r="J15" s="67" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="K15" s="61" t="str">
+        <x:v>C/R</x:v>
       </x:c>
       <x:c r="L15" s="61" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="M15" s="58" t="str">
-        <x:v>C</x:v>
+      <x:c r="M15" s="61" t="str">
+        <x:v>C/R</x:v>
       </x:c>
       <x:c r="N15" s="58" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="37" t="str">
-        <x:v>A-high</x:v>
-      </x:c>
-      <x:c r="B16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="J16" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L16" s="60" t="str">
+      <x:c r="A16" s="50" t="str">
+        <x:v>2 overcards + BDFD</x:v>
+      </x:c>
+      <x:c r="B16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J16" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="L16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="N16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="37" t="str">
+        <x:v>Air</x:v>
+      </x:c>
+      <x:c r="B17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="J17" s="45" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="M16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N16" s="60" t="str">
+      <x:c r="K17" s="60" t="str">
         <x:v>F/C</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="50" t="str">
-        <x:v>A-high + draw</x:v>
-      </x:c>
-      <x:c r="B17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H17" s="67" t="str">
-        <x:v>F/R</x:v>
-      </x:c>
-      <x:c r="I17" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="J17" s="67" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="K17" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="L17" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="M17" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="N17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="37" t="str">
-        <x:v>Air</x:v>
-      </x:c>
-      <x:c r="B18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="H18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="J18" s="45" t="str">
+      <x:c r="L17" s="60" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="K18" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="L18" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="M18" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="N18" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="37" t="str">
-        <x:v>Air + draw</x:v>
-      </x:c>
-      <x:c r="B19" s="45" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="C19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="D19" s="45" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="E19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="F19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H19" s="45" t="str">
-        <x:v>F/R</x:v>
-      </x:c>
-      <x:c r="I19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="J19" s="45" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="K19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="L19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="M19" s="60" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="N19" s="60" t="str">
-        <x:v>C/R</x:v>
+      <x:c r="M17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="N17" s="82" t="str">
+        <x:v>F</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5319,46 +4876,46 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="37" t="str">
         <x:v>Top pair</x:v>
       </x:c>
-      <x:c r="B9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="C9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="D9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J9" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M9" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="N9" s="58" t="str">
+      <x:c r="B9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J9" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="L9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M9" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="N9" s="56" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -5372,16 +4929,16 @@
       <x:c r="C10" s="57" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="D10" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E10" s="84" t="str">
+      <x:c r="D10" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E10" s="82" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="F10" s="45" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="G10" s="84" t="str">
+      <x:c r="G10" s="82" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="H10" s="49" t="str">
@@ -5416,7 +4973,7 @@
       <x:c r="C11" s="56" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D11" s="79" t="str">
+      <x:c r="D11" s="78" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="E11" s="60" t="str">
@@ -5425,7 +4982,7 @@
       <x:c r="F11" s="45" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="G11" s="84" t="str">
+      <x:c r="G11" s="82" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="H11" s="41" t="str">
@@ -5457,19 +5014,19 @@
       <x:c r="B12" s="45" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="C12" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D12" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E12" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F12" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G12" s="84" t="str">
+      <x:c r="C12" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D12" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E12" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F12" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G12" s="82" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="H12" s="45" t="str">
@@ -5498,22 +5055,22 @@
       <x:c r="A13" s="50" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C13" s="83" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E13" s="83" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G13" s="83" t="str">
+      <x:c r="B13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C13" s="81" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E13" s="81" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G13" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="H13" s="51" t="str">
@@ -5522,16 +5079,16 @@
       <x:c r="I13" s="61" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="J13" s="80" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K13" s="83" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L13" s="83" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="M13" s="83" t="str">
+      <x:c r="J13" s="79" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="K13" s="81" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="L13" s="81" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="M13" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="N13" s="61" t="str">
@@ -5540,81 +5097,81 @@
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="37" t="str">
-        <x:v>2 overcards</x:v>
-      </x:c>
-      <x:c r="B14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D14" s="49" t="str">
-        <x:v>—</x:v>
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B14" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D14" s="41" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="E14" s="57" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="F14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I14" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="J14" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="K14" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L14" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="M14" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N14" s="84" t="str">
-        <x:v>F</x:v>
+      <x:c r="F14" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H14" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J14" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="L14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M14" s="56" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="N14" s="56" t="str">
+        <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="50" t="str">
-        <x:v>2 overcards + draw</x:v>
-      </x:c>
-      <x:c r="B15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G15" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J15" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="K15" s="59" t="str">
-        <x:v>—</x:v>
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B15" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C15" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D15" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E15" s="61" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="F15" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G15" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H15" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I15" s="61" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="J15" s="51" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K15" s="58" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="L15" s="58" t="str">
         <x:v>C</x:v>
@@ -5622,184 +5179,96 @@
       <x:c r="M15" s="58" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="N15" s="61" t="str">
+      <x:c r="N15" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="50" t="str">
+        <x:v>2 overcards + BDFD</x:v>
+      </x:c>
+      <x:c r="B16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="J16" s="53" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="K16" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="L16" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M16" s="61" t="str">
         <x:v>F/C</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="37" t="str">
-        <x:v>A-high</x:v>
-      </x:c>
-      <x:c r="B16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G16" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H16" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="J16" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="M16" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N16" s="84" t="str">
+      <x:c r="N16" s="81" t="str">
         <x:v>F</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="50" t="str">
-        <x:v>A-high + draw</x:v>
-      </x:c>
-      <x:c r="B17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F17" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="H17" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I17" s="61" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="J17" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="N17" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="37" t="str">
+      <x:c r="A17" s="37" t="str">
         <x:v>Air</x:v>
       </x:c>
-      <x:c r="B18" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C18" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D18" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E18" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="H18" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="J18" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="L18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="M18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="N18" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="37" t="str">
-        <x:v>Air + draw</x:v>
-      </x:c>
-      <x:c r="B19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="C19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="D19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E19" s="60" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="F19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J19" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M19" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="N19" s="56" t="str">
-        <x:v>C</x:v>
+      <x:c r="B17" s="49" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C17" s="57" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D17" s="49" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E17" s="57" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H17" s="49" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="J17" s="78" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="K17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="L17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="M17" s="82" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="N17" s="82" t="str">
+        <x:v>F</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5828,12 +5297,12 @@
       <x:c r="D1" s="3"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="85" t="str">
+      <x:c r="A2" s="84" t="str">
         <x:v>Методика</x:v>
       </x:c>
-      <x:c r="B2" s="85"/>
-      <x:c r="C2" s="85"/>
-      <x:c r="D2" s="85"/>
+      <x:c r="B2" s="84"/>
+      <x:c r="C2" s="84"/>
+      <x:c r="D2" s="84"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3"/>
@@ -5852,108 +5321,112 @@
       <x:c r="D4" s="21"/>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
-      <x:c r="A5" s="86" t="str">
+      <x:c r="A5" s="85" t="str">
         <x:v>Флопы</x:v>
       </x:c>
-      <x:c r="B5" s="86" t="str">
+      <x:c r="B5" s="85" t="str">
         <x:v>286 canonical unpaired rainbow flops, B13: 13 взаимоисключающих категорий</x:v>
       </x:c>
       <x:c r="C5" s="3"/>
       <x:c r="D5" s="3"/>
     </x:row>
     <x:row r="6" ht="27" customHeight="1">
-      <x:c r="A6" s="86" t="str">
+      <x:c r="A6" s="85" t="str">
         <x:v>Частоты</x:v>
       </x:c>
-      <x:c r="B6" s="86" t="str">
+      <x:c r="B6" s="85" t="str">
         <x:v>Равное среднее по concrete combo на флопе, затем равное среднее по реальным флопам категории</x:v>
       </x:c>
       <x:c r="C6" s="3"/>
       <x:c r="D6" s="3"/>
     </x:row>
     <x:row r="7" ht="27" customHeight="1">
-      <x:c r="A7" s="86" t="str">
+      <x:c r="A7" s="85" t="str">
         <x:v>Чистое действие</x:v>
       </x:c>
-      <x:c r="B7" s="86" t="str">
+      <x:c r="B7" s="85" t="str">
         <x:v>Наибольшая средняя частота строго &gt;65%</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3"/>
     </x:row>
     <x:row r="8" ht="27" customHeight="1">
-      <x:c r="A8" s="86" t="str">
+      <x:c r="A8" s="85" t="str">
         <x:v>Микс</x:v>
       </x:c>
-      <x:c r="B8" s="86" t="str">
+      <x:c r="B8" s="85" t="str">
         <x:v>Иначе два наиболее частых действия, строго 50/50</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
       <x:c r="D8" s="3"/>
     </x:row>
     <x:row r="9" ht="27" customHeight="1">
-      <x:c r="A9" s="86" t="str">
+      <x:c r="A9" s="85" t="str">
         <x:v>Вес диапазона</x:v>
       </x:c>
-      <x:c r="B9" s="86" t="str">
+      <x:c r="B9" s="85" t="str">
         <x:v>Combo с reach_probability &gt;0 участвует независимо от величины reach</x:v>
       </x:c>
       <x:c r="C9" s="3"/>
       <x:c r="D9" s="3"/>
     </x:row>
     <x:row r="10" ht="27" customHeight="1">
-      <x:c r="A10" s="86" t="str">
+      <x:c r="A10" s="85" t="str">
         <x:v>EV-аудит</x:v>
       </x:c>
-      <x:c r="B10" s="86" t="str">
+      <x:c r="B10" s="85" t="str">
         <x:v>Reach-weighted local regret против solved opponent; не adaptive exploitability</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
     </x:row>
     <x:row r="11" ht="27" customHeight="1">
-      <x:c r="A11" s="86" t="str">
+      <x:c r="A11" s="85" t="str">
         <x:v>Категории рук</x:v>
       </x:c>
-      <x:c r="B11" s="86" t="str">
-        <x:v>Те же 13 категорий и те же правила BDFD/Gutshot/OESD</x:v>
+      <x:c r="B11" s="85" t="str">
+        <x:v>7 made-категорий; затем OESD; Gutshot; 2 overcards + BDFD; Air</x:v>
       </x:c>
       <x:c r="C11" s="3"/>
       <x:c r="D11" s="3"/>
     </x:row>
     <x:row r="12" ht="27" customHeight="1">
-      <x:c r="A12" s="86" t="str">
-        <x:v>Категории флопов</x:v>
-      </x:c>
-      <x:c r="B12" s="86" t="str">
-        <x:v>B13 — итоговые категории этой таблицы</x:v>
+      <x:c r="A12" s="85" t="str">
+        <x:v>Приоритет неготовых</x:v>
+      </x:c>
+      <x:c r="B12" s="85" t="str">
+        <x:v>OESD &gt; Gutshot &gt; 2 overcards + BDFD &gt; Air; BDFD без двух оверкарт уходит в Air</x:v>
       </x:c>
       <x:c r="C12" s="3"/>
       <x:c r="D12" s="3"/>
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
-      <x:c r="A13" s="86" t="str">
-        <x:v>Роль исходной B13</x:v>
-      </x:c>
-      <x:c r="B13" s="86" t="str">
-        <x:v>Итоговые столбцы стратегии</x:v>
+      <x:c r="A13" s="85" t="str">
+        <x:v>Категории флопов</x:v>
+      </x:c>
+      <x:c r="B13" s="85" t="str">
+        <x:v>B13 — итоговые категории этой таблицы</x:v>
       </x:c>
       <x:c r="C13" s="3"/>
       <x:c r="D13" s="3"/>
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
-      <x:c r="A14" s="86" t="str">
-        <x:v>JT9</x:v>
-      </x:c>
-      <x:c r="B14" s="86" t="str">
-        <x:v>Исходная B13 = [J-8]x con; в 8-групповой таблице = Middle connected</x:v>
+      <x:c r="A14" s="85" t="str">
+        <x:v>Роль исходной B13</x:v>
+      </x:c>
+      <x:c r="B14" s="85" t="str">
+        <x:v>Итоговые столбцы стратегии</x:v>
       </x:c>
       <x:c r="C14" s="3"/>
       <x:c r="D14" s="3"/>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
-      <x:c r="A15" s="3"/>
-      <x:c r="B15" s="3"/>
+      <x:c r="A15" s="85" t="str">
+        <x:v>JT9</x:v>
+      </x:c>
+      <x:c r="B15" s="85" t="str">
+        <x:v>Исходная B13 = [J-8]x con; в 8-групповой таблице = Middle connected</x:v>
+      </x:c>
       <x:c r="C15" s="3"/>
       <x:c r="D15" s="3"/>
     </x:row>
@@ -5964,192 +5437,198 @@
       <x:c r="D16" s="3"/>
     </x:row>
     <x:row r="17" ht="27" customHeight="1">
-      <x:c r="A17" s="87" t="str">
+      <x:c r="A17" s="3"/>
+      <x:c r="B17" s="3"/>
+      <x:c r="C17" s="3"/>
+      <x:c r="D17" s="3"/>
+    </x:row>
+    <x:row r="18" ht="27" customHeight="1">
+      <x:c r="A18" s="86" t="str">
         <x:v>Категория флопов</x:v>
       </x:c>
-      <x:c r="B17" s="87" t="str">
+      <x:c r="B18" s="86" t="str">
         <x:v>Входящие B13 / определение</x:v>
       </x:c>
-      <x:c r="C17" s="87" t="str">
+      <x:c r="C18" s="86" t="str">
         <x:v>Количество</x:v>
       </x:c>
-      <x:c r="D17" s="87" t="str">
+      <x:c r="D18" s="86" t="str">
         <x:v>Пояснение</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="27" customHeight="1">
-      <x:c r="A18" s="90" t="str">
+    <x:row r="19" ht="27" customHeight="1">
+      <x:c r="A19" s="89" t="str">
         <x:v>ABB</x:v>
       </x:c>
-      <x:c r="B18" s="90" t="str">
+      <x:c r="B19" s="89" t="str">
         <x:v>A + две broadway-карты</x:v>
       </x:c>
-      <x:c r="C18" s="91" t="n">
+      <x:c r="C19" s="90" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D18" s="90" t="str">
+      <x:c r="D19" s="89" t="str">
         <x:v>B = T/J/Q/K; A отдельно</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="27" customHeight="1">
-      <x:c r="A19" s="90" t="str">
+    <x:row r="20" ht="27" customHeight="1">
+      <x:c r="A20" s="89" t="str">
         <x:v>A[K/Q]x</x:v>
       </x:c>
-      <x:c r="B19" s="90" t="str">
+      <x:c r="B20" s="89" t="str">
         <x:v>A + K/Q + карта 9 и ниже</x:v>
       </x:c>
-      <x:c r="C19" s="91" t="n">
+      <x:c r="C20" s="90" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="D19" s="90" t="str">
+      <x:c r="D20" s="89" t="str">
         <x:v>ABB исключён</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="27" customHeight="1">
-      <x:c r="A20" s="90" t="str">
+    <x:row r="21" ht="27" customHeight="1">
+      <x:c r="A21" s="89" t="str">
         <x:v>A[J-T][9-5]</x:v>
       </x:c>
-      <x:c r="B20" s="90" t="str">
+      <x:c r="B21" s="89" t="str">
         <x:v>A + J/T + карта 9…5</x:v>
       </x:c>
-      <x:c r="C20" s="91" t="n">
+      <x:c r="C21" s="90" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D20" s="90" t="str"/>
-    </x:row>
-    <x:row r="21" ht="27" customHeight="1">
-      <x:c r="A21" s="90" t="str">
+      <x:c r="D21" s="89" t="str"/>
+    </x:row>
+    <x:row r="22" ht="27" customHeight="1">
+      <x:c r="A22" s="89" t="str">
         <x:v>A[J-T][4-2]</x:v>
       </x:c>
-      <x:c r="B21" s="90" t="str">
+      <x:c r="B22" s="89" t="str">
         <x:v>A + J/T + карта 4…2</x:v>
       </x:c>
-      <x:c r="C21" s="91" t="n">
+      <x:c r="C22" s="90" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D21" s="90" t="str"/>
-    </x:row>
-    <x:row r="22" ht="27" customHeight="1">
-      <x:c r="A22" s="90" t="str">
+      <x:c r="D22" s="89" t="str"/>
+    </x:row>
+    <x:row r="23" ht="27" customHeight="1">
+      <x:c r="A23" s="89" t="str">
         <x:v>A[9-7]x</x:v>
       </x:c>
-      <x:c r="B22" s="90" t="str">
+      <x:c r="B23" s="89" t="str">
         <x:v>A + 9/8/7 + более низкая</x:v>
       </x:c>
-      <x:c r="C22" s="91" t="n">
+      <x:c r="C23" s="90" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="D22" s="90" t="str"/>
-    </x:row>
-    <x:row r="23" ht="27" customHeight="1">
-      <x:c r="A23" s="90" t="str">
+      <x:c r="D23" s="89" t="str"/>
+    </x:row>
+    <x:row r="24" ht="27" customHeight="1">
+      <x:c r="A24" s="89" t="str">
         <x:v>A[6-2]x</x:v>
       </x:c>
-      <x:c r="B23" s="90" t="str">
+      <x:c r="B24" s="89" t="str">
         <x:v>A + 6…3 + более низкая</x:v>
       </x:c>
-      <x:c r="C23" s="91" t="n">
+      <x:c r="C24" s="90" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D23" s="90" t="str"/>
-    </x:row>
-    <x:row r="24" ht="27" customHeight="1">
-      <x:c r="A24" s="90" t="str">
+      <x:c r="D24" s="89" t="str"/>
+    </x:row>
+    <x:row r="25" ht="27" customHeight="1">
+      <x:c r="A25" s="89" t="str">
         <x:v>BBB</x:v>
       </x:c>
-      <x:c r="B24" s="90" t="str">
+      <x:c r="B25" s="89" t="str">
         <x:v>Без A; три broadway-карты</x:v>
       </x:c>
-      <x:c r="C24" s="91" t="n">
+      <x:c r="C25" s="90" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D24" s="90" t="str"/>
-    </x:row>
-    <x:row r="25" ht="27" customHeight="1">
-      <x:c r="A25" s="90" t="str">
+      <x:c r="D25" s="89" t="str"/>
+    </x:row>
+    <x:row r="26" ht="27" customHeight="1">
+      <x:c r="A26" s="89" t="str">
         <x:v>BBx</x:v>
       </x:c>
-      <x:c r="B25" s="90" t="str">
+      <x:c r="B26" s="89" t="str">
         <x:v>Без A; две broadway + карта ≤9</x:v>
       </x:c>
-      <x:c r="C25" s="91" t="n">
+      <x:c r="C26" s="90" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="D25" s="90" t="str">
+      <x:c r="D26" s="89" t="str">
         <x:v>JT9 исключён</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="27" customHeight="1">
-      <x:c r="A26" s="90" t="str">
+    <x:row r="27" ht="27" customHeight="1">
+      <x:c r="A27" s="89" t="str">
         <x:v>K/Qx dis</x:v>
       </x:c>
-      <x:c r="B26" s="90" t="str">
+      <x:c r="B27" s="89" t="str">
         <x:v>Старшая K/Q; lower gap &gt;1</x:v>
       </x:c>
-      <x:c r="C26" s="91" t="n">
+      <x:c r="C27" s="90" t="n">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="D26" s="90" t="str">
+      <x:c r="D27" s="89" t="str">
         <x:v>Не BBx</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="27" customHeight="1">
-      <x:c r="A27" s="90" t="str">
+    <x:row r="28" ht="27" customHeight="1">
+      <x:c r="A28" s="89" t="str">
         <x:v>K/Qx con</x:v>
       </x:c>
-      <x:c r="B27" s="90" t="str">
+      <x:c r="B28" s="89" t="str">
         <x:v>Старшая K/Q; lower gap =1</x:v>
       </x:c>
-      <x:c r="C27" s="91" t="n">
+      <x:c r="C28" s="90" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="D27" s="90" t="str">
+      <x:c r="D28" s="89" t="str">
         <x:v>Не BBx</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="27" customHeight="1">
-      <x:c r="A28" s="90" t="str">
+    <x:row r="29" ht="27" customHeight="1">
+      <x:c r="A29" s="89" t="str">
         <x:v>[J-8]x dis</x:v>
       </x:c>
-      <x:c r="B28" s="90" t="str">
+      <x:c r="B29" s="89" t="str">
         <x:v>Старшая J/T/9/8; lower gap &gt;1</x:v>
       </x:c>
-      <x:c r="C28" s="91" t="n">
+      <x:c r="C29" s="90" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="D28" s="90" t="str"/>
-    </x:row>
-    <x:row r="29" ht="27" customHeight="1">
-      <x:c r="A29" s="90" t="str">
+      <x:c r="D29" s="89" t="str"/>
+    </x:row>
+    <x:row r="30" ht="27" customHeight="1">
+      <x:c r="A30" s="89" t="str">
         <x:v>[J-8]x con</x:v>
       </x:c>
-      <x:c r="B29" s="90" t="str">
+      <x:c r="B30" s="89" t="str">
         <x:v>Старшая J/T/9/8; lower gap =1</x:v>
       </x:c>
-      <x:c r="C29" s="91" t="n">
+      <x:c r="C30" s="90" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D29" s="90" t="str">
+      <x:c r="D30" s="89" t="str">
         <x:v>Включает JT9</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="27" customHeight="1">
-      <x:c r="A30" s="90" t="str">
+    <x:row r="31" ht="27" customHeight="1">
+      <x:c r="A31" s="89" t="str">
         <x:v>[7-4]x</x:v>
       </x:c>
-      <x:c r="B30" s="90" t="str">
+      <x:c r="B31" s="89" t="str">
         <x:v>Старшая карта 7 или ниже</x:v>
       </x:c>
-      <x:c r="C30" s="91" t="n">
+      <x:c r="C31" s="90" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D30" s="90" t="str"/>
-    </x:row>
-    <x:row r="31" ht="27" customHeight="1">
-      <x:c r="A31" s="3"/>
-      <x:c r="B31" s="3"/>
-      <x:c r="C31" s="3"/>
-      <x:c r="D31" s="3"/>
+      <x:c r="D31" s="89" t="str"/>
+    </x:row>
+    <x:row r="32" ht="27" customHeight="1">
+      <x:c r="A32" s="3"/>
+      <x:c r="B32" s="3"/>
+      <x:c r="C32" s="3"/>
+      <x:c r="D32" s="3"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Order mixed actions by solver frequency
</commit_message>
<xml_diff>
--- a/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_simplified_flop_strategy.xlsx
+++ b/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_simplified_flop_strategy.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R69ec1f52de3345c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="Rd5c42a3f64dc40f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="R780dc711b1514677"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="Rde145329db484f57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R4dc32074d93e4a13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="R4364952ff6c5439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="R5e0981b401044771"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="8" r:id="Re844cf4617ea4045"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd981b58a5f554001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="R58684e9fdd244079"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="Rb9d8686122c14646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="R3dd2a38668a74b11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R783364362681451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="R6a0ab33709c64092"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="R62a8b3cf99934870"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="8" r:id="Rd84cfcf40b6b4b67"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1493,7 +1493,7 @@
         <x:v>X</x:v>
       </x:c>
       <x:c r="N7" s="60" t="str">
-        <x:v>X/D</x:v>
+        <x:v>D/X</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
@@ -1757,7 +1757,7 @@
         <x:v>X</x:v>
       </x:c>
       <x:c r="N13" s="61" t="str">
-        <x:v>X/D</x:v>
+        <x:v>D/X</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
@@ -1801,7 +1801,7 @@
         <x:v>X</x:v>
       </x:c>
       <x:c r="N14" s="60" t="str">
-        <x:v>X/D</x:v>
+        <x:v>D/X</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
@@ -1889,7 +1889,7 @@
         <x:v>X</x:v>
       </x:c>
       <x:c r="N16" s="61" t="str">
-        <x:v>X/D</x:v>
+        <x:v>D/X</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
@@ -2204,7 +2204,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="N8" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
@@ -2218,7 +2218,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D9" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="E9" s="60" t="str">
         <x:v>X/B</x:v>
@@ -2236,16 +2236,16 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="J9" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="K9" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
       <x:c r="L9" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="M9" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="N9" s="69" t="str">
         <x:v>B</x:v>
@@ -2277,7 +2277,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="I10" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="J10" s="41" t="str">
         <x:v>X</x:v>
@@ -2303,10 +2303,10 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C11" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="D11" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="E11" s="56" t="str">
         <x:v>X</x:v>
@@ -2318,7 +2318,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="H11" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="I11" s="60" t="str">
         <x:v>X/B</x:v>
@@ -2330,10 +2330,10 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="L11" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="M11" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="N11" s="69" t="str">
         <x:v>B</x:v>
@@ -2362,25 +2362,25 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="H12" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="I12" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="J12" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="K12" s="56" t="str">
         <x:v>X</x:v>
       </x:c>
       <x:c r="L12" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="M12" s="56" t="str">
         <x:v>X</x:v>
       </x:c>
       <x:c r="N12" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
@@ -2391,13 +2391,13 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C13" s="61" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="D13" s="67" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="E13" s="61" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="F13" s="67" t="str">
         <x:v>X/B</x:v>
@@ -2409,7 +2409,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="I13" s="61" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="J13" s="51" t="str">
         <x:v>X</x:v>
@@ -2512,7 +2512,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="N15" s="61" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
@@ -2564,7 +2564,7 @@
         <x:v>Air</x:v>
       </x:c>
       <x:c r="B17" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="C17" s="60" t="str">
         <x:v>X/B</x:v>
@@ -2573,28 +2573,28 @@
         <x:v>X/B</x:v>
       </x:c>
       <x:c r="E17" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="F17" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="G17" s="60" t="str">
         <x:v>X/B</x:v>
       </x:c>
       <x:c r="H17" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="I17" s="69" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="J17" s="45" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="K17" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="L17" s="60" t="str">
-        <x:v>X/B</x:v>
+        <x:v>B/X</x:v>
       </x:c>
       <x:c r="M17" s="60" t="str">
         <x:v>X/B</x:v>
@@ -2791,7 +2791,7 @@
         <x:v>Two pair+</x:v>
       </x:c>
       <x:c r="B7" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="C7" s="80" t="str">
         <x:v>R</x:v>
@@ -2929,10 +2929,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="D10" s="45" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="E10" s="60" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="F10" s="41" t="str">
         <x:v>C</x:v>
@@ -2967,13 +2967,13 @@
         <x:v>Second pair</x:v>
       </x:c>
       <x:c r="B11" s="45" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="C11" s="56" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="D11" s="45" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="E11" s="56" t="str">
         <x:v>C</x:v>
@@ -3011,7 +3011,7 @@
         <x:v>Third pair</x:v>
       </x:c>
       <x:c r="B12" s="45" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="C12" s="60" t="str">
         <x:v>F/C</x:v>
@@ -3020,7 +3020,7 @@
         <x:v>F/C</x:v>
       </x:c>
       <x:c r="E12" s="60" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="F12" s="41" t="str">
         <x:v>C</x:v>
@@ -3029,7 +3029,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="H12" s="45" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="I12" s="60" t="str">
         <x:v>C/R</x:v>
@@ -3070,7 +3070,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="G13" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="H13" s="79" t="str">
         <x:v>F</x:v>
@@ -3099,7 +3099,7 @@
         <x:v>OESD</x:v>
       </x:c>
       <x:c r="B14" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="C14" s="60" t="str">
         <x:v>C/R</x:v>
@@ -3117,10 +3117,10 @@
         <x:v>R</x:v>
       </x:c>
       <x:c r="H14" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="I14" s="60" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="J14" s="74" t="str">
         <x:v>R</x:v>
@@ -3155,7 +3155,7 @@
         <x:v>C/R</x:v>
       </x:c>
       <x:c r="F15" s="67" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="G15" s="61" t="str">
         <x:v>C/R</x:v>
@@ -3164,22 +3164,22 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="I15" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="J15" s="67" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="K15" s="61" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="L15" s="61" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="M15" s="61" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="N15" s="61" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
@@ -3223,7 +3223,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="N16" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
@@ -3599,7 +3599,7 @@
         <x:v>F/C</x:v>
       </x:c>
       <x:c r="E10" s="60" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="F10" s="41" t="str">
         <x:v>C</x:v>
@@ -3643,7 +3643,7 @@
         <x:v>F/C</x:v>
       </x:c>
       <x:c r="E11" s="60" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="F11" s="41" t="str">
         <x:v>C</x:v>
@@ -3652,7 +3652,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="H11" s="45" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="I11" s="56" t="str">
         <x:v>C</x:v>
@@ -3752,7 +3752,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="L13" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="M13" s="81" t="str">
         <x:v>F</x:v>
@@ -3784,7 +3784,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="H14" s="45" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="I14" s="56" t="str">
         <x:v>C</x:v>
@@ -3810,7 +3810,7 @@
         <x:v>Gutshot</x:v>
       </x:c>
       <x:c r="B15" s="67" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="C15" s="58" t="str">
         <x:v>C</x:v>
@@ -3819,7 +3819,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="E15" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="F15" s="51" t="str">
         <x:v>C</x:v>
@@ -3831,7 +3831,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="I15" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="J15" s="51" t="str">
         <x:v>C</x:v>
@@ -4137,13 +4137,13 @@
         <x:v>R</x:v>
       </x:c>
       <x:c r="F7" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="G7" s="60" t="str">
         <x:v>C/R</x:v>
       </x:c>
       <x:c r="H7" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="I7" s="80" t="str">
         <x:v>R</x:v>
@@ -4213,7 +4213,7 @@
         <x:v>Top pair</x:v>
       </x:c>
       <x:c r="B9" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="C9" s="60" t="str">
         <x:v>C/R</x:v>
@@ -4257,7 +4257,7 @@
         <x:v>Underpair</x:v>
       </x:c>
       <x:c r="B10" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="C10" s="56" t="str">
         <x:v>C</x:v>
@@ -4304,22 +4304,22 @@
         <x:v>C/R</x:v>
       </x:c>
       <x:c r="C11" s="60" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="D11" s="45" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="E11" s="60" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="F11" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="G11" s="60" t="str">
         <x:v>C/R</x:v>
       </x:c>
       <x:c r="H11" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="I11" s="60" t="str">
         <x:v>C/R</x:v>
@@ -4345,31 +4345,31 @@
         <x:v>Third pair</x:v>
       </x:c>
       <x:c r="B12" s="45" t="str">
-        <x:v>F/R</x:v>
+        <x:v>R/F</x:v>
       </x:c>
       <x:c r="C12" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="D12" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="E12" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="F12" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="G12" s="60" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="H12" s="45" t="str">
-        <x:v>F/R</x:v>
+        <x:v>R/F</x:v>
       </x:c>
       <x:c r="I12" s="60" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="J12" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="K12" s="60" t="str">
         <x:v>C/R</x:v>
@@ -4401,7 +4401,7 @@
         <x:v>F/C</x:v>
       </x:c>
       <x:c r="F13" s="67" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="G13" s="58" t="str">
         <x:v>C</x:v>
@@ -4416,7 +4416,7 @@
         <x:v>C/R</x:v>
       </x:c>
       <x:c r="K13" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="L13" s="58" t="str">
         <x:v>C</x:v>
@@ -4433,13 +4433,13 @@
         <x:v>OESD</x:v>
       </x:c>
       <x:c r="B14" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="C14" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="D14" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="E14" s="57" t="str">
         <x:v>—</x:v>
@@ -4451,16 +4451,16 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="H14" s="45" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="I14" s="60" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="J14" s="74" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="K14" s="60" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="L14" s="80" t="str">
         <x:v>R</x:v>
@@ -4469,7 +4469,7 @@
         <x:v>R</x:v>
       </x:c>
       <x:c r="N14" s="60" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
@@ -4477,13 +4477,13 @@
         <x:v>Gutshot</x:v>
       </x:c>
       <x:c r="B15" s="67" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="C15" s="61" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="D15" s="67" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="E15" s="61" t="str">
         <x:v>C/R</x:v>
@@ -4498,7 +4498,7 @@
         <x:v>F/R</x:v>
       </x:c>
       <x:c r="I15" s="61" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="J15" s="67" t="str">
         <x:v>C/R</x:v>
@@ -4507,7 +4507,7 @@
         <x:v>C/R</x:v>
       </x:c>
       <x:c r="L15" s="61" t="str">
-        <x:v>C/R</x:v>
+        <x:v>R/C</x:v>
       </x:c>
       <x:c r="M15" s="61" t="str">
         <x:v>C/R</x:v>
@@ -4951,7 +4951,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="K10" s="60" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="L10" s="56" t="str">
         <x:v>C</x:v>
@@ -4980,7 +4980,7 @@
         <x:v>F/C</x:v>
       </x:c>
       <x:c r="F11" s="45" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="G11" s="82" t="str">
         <x:v>F</x:v>
@@ -5033,7 +5033,7 @@
         <x:v>F/C</x:v>
       </x:c>
       <x:c r="I12" s="60" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="J12" s="41" t="str">
         <x:v>C</x:v>
@@ -5077,7 +5077,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="I13" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="J13" s="79" t="str">
         <x:v>F</x:v>
@@ -5153,7 +5153,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="E15" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="F15" s="51" t="str">
         <x:v>C</x:v>
@@ -5165,7 +5165,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="I15" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="J15" s="51" t="str">
         <x:v>C</x:v>
@@ -5221,7 +5221,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="M16" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="N16" s="81" t="str">
         <x:v>F</x:v>
@@ -5332,107 +5332,111 @@
     </x:row>
     <x:row r="6" ht="27" customHeight="1">
       <x:c r="A6" s="85" t="str">
-        <x:v>Частоты</x:v>
+        <x:v>Диапазоны</x:v>
       </x:c>
       <x:c r="B6" s="85" t="str">
-        <x:v>Равное среднее по concrete combo на флопе, затем равное среднее по реальным флопам категории</x:v>
+        <x:v>RNG001: UTG open 2.5 bb / BB call из библиотеки TexasSolverGPU v0.2.0</x:v>
       </x:c>
       <x:c r="C6" s="3"/>
       <x:c r="D6" s="3"/>
     </x:row>
     <x:row r="7" ht="27" customHeight="1">
       <x:c r="A7" s="85" t="str">
-        <x:v>Чистое действие</x:v>
+        <x:v>Частоты</x:v>
       </x:c>
       <x:c r="B7" s="85" t="str">
-        <x:v>Наибольшая средняя частота строго &gt;65%</x:v>
+        <x:v>Равное среднее по concrete combo на флопе, затем равное среднее по реальным флопам категории</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3"/>
     </x:row>
     <x:row r="8" ht="27" customHeight="1">
       <x:c r="A8" s="85" t="str">
-        <x:v>Микс</x:v>
+        <x:v>Чистое действие</x:v>
       </x:c>
       <x:c r="B8" s="85" t="str">
-        <x:v>Иначе два наиболее частых действия, строго 50/50</x:v>
+        <x:v>Наибольшая средняя частота строго &gt;65%</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
       <x:c r="D8" s="3"/>
     </x:row>
     <x:row r="9" ht="27" customHeight="1">
       <x:c r="A9" s="85" t="str">
-        <x:v>Вес диапазона</x:v>
+        <x:v>Микс</x:v>
       </x:c>
       <x:c r="B9" s="85" t="str">
-        <x:v>Combo с reach_probability &gt;0 участвует независимо от величины reach</x:v>
+        <x:v>Иначе два наиболее частых действия, строго 50/50; первым указано более частое действие солвера</x:v>
       </x:c>
       <x:c r="C9" s="3"/>
       <x:c r="D9" s="3"/>
     </x:row>
     <x:row r="10" ht="27" customHeight="1">
       <x:c r="A10" s="85" t="str">
-        <x:v>EV-аудит</x:v>
+        <x:v>Вес диапазона</x:v>
       </x:c>
       <x:c r="B10" s="85" t="str">
-        <x:v>Reach-weighted local regret против solved opponent; не adaptive exploitability</x:v>
+        <x:v>Combo с reach_probability &gt;0 участвует независимо от величины reach</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
     </x:row>
     <x:row r="11" ht="27" customHeight="1">
       <x:c r="A11" s="85" t="str">
-        <x:v>Категории рук</x:v>
+        <x:v>EV-аудит</x:v>
       </x:c>
       <x:c r="B11" s="85" t="str">
-        <x:v>7 made-категорий; затем OESD; Gutshot; 2 overcards + BDFD; Air</x:v>
+        <x:v>Reach-weighted local regret против solved opponent; не adaptive exploitability</x:v>
       </x:c>
       <x:c r="C11" s="3"/>
       <x:c r="D11" s="3"/>
     </x:row>
     <x:row r="12" ht="27" customHeight="1">
       <x:c r="A12" s="85" t="str">
-        <x:v>Приоритет неготовых</x:v>
+        <x:v>Категории рук</x:v>
       </x:c>
       <x:c r="B12" s="85" t="str">
-        <x:v>OESD &gt; Gutshot &gt; 2 overcards + BDFD &gt; Air; BDFD без двух оверкарт уходит в Air</x:v>
+        <x:v>7 made-категорий; затем OESD; Gutshot; 2 overcards + BDFD; Air</x:v>
       </x:c>
       <x:c r="C12" s="3"/>
       <x:c r="D12" s="3"/>
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
       <x:c r="A13" s="85" t="str">
-        <x:v>Категории флопов</x:v>
+        <x:v>Приоритет неготовых</x:v>
       </x:c>
       <x:c r="B13" s="85" t="str">
-        <x:v>B13 — итоговые категории этой таблицы</x:v>
+        <x:v>OESD &gt; Gutshot &gt; 2 overcards + BDFD &gt; Air; BDFD без двух оверкарт уходит в Air</x:v>
       </x:c>
       <x:c r="C13" s="3"/>
       <x:c r="D13" s="3"/>
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
       <x:c r="A14" s="85" t="str">
-        <x:v>Роль исходной B13</x:v>
+        <x:v>Категории флопов</x:v>
       </x:c>
       <x:c r="B14" s="85" t="str">
-        <x:v>Итоговые столбцы стратегии</x:v>
+        <x:v>B13 — итоговые категории этой таблицы</x:v>
       </x:c>
       <x:c r="C14" s="3"/>
       <x:c r="D14" s="3"/>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
       <x:c r="A15" s="85" t="str">
-        <x:v>JT9</x:v>
+        <x:v>Роль исходной B13</x:v>
       </x:c>
       <x:c r="B15" s="85" t="str">
-        <x:v>Исходная B13 = [J-8]x con; в 8-групповой таблице = Middle connected</x:v>
+        <x:v>Итоговые столбцы стратегии</x:v>
       </x:c>
       <x:c r="C15" s="3"/>
       <x:c r="D15" s="3"/>
     </x:row>
     <x:row r="16" ht="27" customHeight="1">
-      <x:c r="A16" s="3"/>
-      <x:c r="B16" s="3"/>
+      <x:c r="A16" s="85" t="str">
+        <x:v>JT9</x:v>
+      </x:c>
+      <x:c r="B16" s="85" t="str">
+        <x:v>Исходная B13 = [J-8]x con; в 8-групповой таблице = Middle connected</x:v>
+      </x:c>
       <x:c r="C16" s="3"/>
       <x:c r="D16" s="3"/>
     </x:row>
@@ -5443,144 +5447,136 @@
       <x:c r="D17" s="3"/>
     </x:row>
     <x:row r="18" ht="27" customHeight="1">
-      <x:c r="A18" s="86" t="str">
+      <x:c r="A18" s="3"/>
+      <x:c r="B18" s="3"/>
+      <x:c r="C18" s="3"/>
+      <x:c r="D18" s="3"/>
+    </x:row>
+    <x:row r="19" ht="27" customHeight="1">
+      <x:c r="A19" s="86" t="str">
         <x:v>Категория флопов</x:v>
       </x:c>
-      <x:c r="B18" s="86" t="str">
+      <x:c r="B19" s="86" t="str">
         <x:v>Входящие B13 / определение</x:v>
       </x:c>
-      <x:c r="C18" s="86" t="str">
+      <x:c r="C19" s="86" t="str">
         <x:v>Количество</x:v>
       </x:c>
-      <x:c r="D18" s="86" t="str">
+      <x:c r="D19" s="86" t="str">
         <x:v>Пояснение</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="27" customHeight="1">
-      <x:c r="A19" s="89" t="str">
-        <x:v>ABB</x:v>
-      </x:c>
-      <x:c r="B19" s="89" t="str">
-        <x:v>A + две broadway-карты</x:v>
-      </x:c>
-      <x:c r="C19" s="90" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D19" s="89" t="str">
-        <x:v>B = T/J/Q/K; A отдельно</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="27" customHeight="1">
       <x:c r="A20" s="89" t="str">
-        <x:v>A[K/Q]x</x:v>
+        <x:v>ABB</x:v>
       </x:c>
       <x:c r="B20" s="89" t="str">
-        <x:v>A + K/Q + карта 9 и ниже</x:v>
+        <x:v>A + две broadway-карты</x:v>
       </x:c>
       <x:c r="C20" s="90" t="n">
-        <x:v>16</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D20" s="89" t="str">
-        <x:v>ABB исключён</x:v>
+        <x:v>B = T/J/Q/K; A отдельно</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="27" customHeight="1">
       <x:c r="A21" s="89" t="str">
-        <x:v>A[J-T][9-5]</x:v>
+        <x:v>A[K/Q]x</x:v>
       </x:c>
       <x:c r="B21" s="89" t="str">
-        <x:v>A + J/T + карта 9…5</x:v>
+        <x:v>A + K/Q + карта 9 и ниже</x:v>
       </x:c>
       <x:c r="C21" s="90" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D21" s="89" t="str"/>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D21" s="89" t="str">
+        <x:v>ABB исключён</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="27" customHeight="1">
       <x:c r="A22" s="89" t="str">
-        <x:v>A[J-T][4-2]</x:v>
+        <x:v>A[J-T][9-5]</x:v>
       </x:c>
       <x:c r="B22" s="89" t="str">
-        <x:v>A + J/T + карта 4…2</x:v>
+        <x:v>A + J/T + карта 9…5</x:v>
       </x:c>
       <x:c r="C22" s="90" t="n">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D22" s="89" t="str"/>
     </x:row>
     <x:row r="23" ht="27" customHeight="1">
       <x:c r="A23" s="89" t="str">
-        <x:v>A[9-7]x</x:v>
+        <x:v>A[J-T][4-2]</x:v>
       </x:c>
       <x:c r="B23" s="89" t="str">
-        <x:v>A + 9/8/7 + более низкая</x:v>
+        <x:v>A + J/T + карта 4…2</x:v>
       </x:c>
       <x:c r="C23" s="90" t="n">
-        <x:v>18</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D23" s="89" t="str"/>
     </x:row>
     <x:row r="24" ht="27" customHeight="1">
       <x:c r="A24" s="89" t="str">
-        <x:v>A[6-2]x</x:v>
+        <x:v>A[9-7]x</x:v>
       </x:c>
       <x:c r="B24" s="89" t="str">
-        <x:v>A + 6…3 + более низкая</x:v>
+        <x:v>A + 9/8/7 + более низкая</x:v>
       </x:c>
       <x:c r="C24" s="90" t="n">
-        <x:v>10</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D24" s="89" t="str"/>
     </x:row>
     <x:row r="25" ht="27" customHeight="1">
       <x:c r="A25" s="89" t="str">
-        <x:v>BBB</x:v>
+        <x:v>A[6-2]x</x:v>
       </x:c>
       <x:c r="B25" s="89" t="str">
-        <x:v>Без A; три broadway-карты</x:v>
+        <x:v>A + 6…3 + более низкая</x:v>
       </x:c>
       <x:c r="C25" s="90" t="n">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D25" s="89" t="str"/>
     </x:row>
     <x:row r="26" ht="27" customHeight="1">
       <x:c r="A26" s="89" t="str">
-        <x:v>BBx</x:v>
+        <x:v>BBB</x:v>
       </x:c>
       <x:c r="B26" s="89" t="str">
-        <x:v>Без A; две broadway + карта ≤9</x:v>
+        <x:v>Без A; три broadway-карты</x:v>
       </x:c>
       <x:c r="C26" s="90" t="n">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="D26" s="89" t="str">
-        <x:v>JT9 исключён</x:v>
-      </x:c>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D26" s="89" t="str"/>
     </x:row>
     <x:row r="27" ht="27" customHeight="1">
       <x:c r="A27" s="89" t="str">
-        <x:v>K/Qx dis</x:v>
+        <x:v>BBx</x:v>
       </x:c>
       <x:c r="B27" s="89" t="str">
-        <x:v>Старшая K/Q; lower gap &gt;1</x:v>
+        <x:v>Без A; две broadway + карта ≤9</x:v>
       </x:c>
       <x:c r="C27" s="90" t="n">
-        <x:v>42</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D27" s="89" t="str">
-        <x:v>Не BBx</x:v>
+        <x:v>JT9 исключён</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="27" customHeight="1">
       <x:c r="A28" s="89" t="str">
-        <x:v>K/Qx con</x:v>
+        <x:v>K/Qx dis</x:v>
       </x:c>
       <x:c r="B28" s="89" t="str">
-        <x:v>Старшая K/Q; lower gap =1</x:v>
+        <x:v>Старшая K/Q; lower gap &gt;1</x:v>
       </x:c>
       <x:c r="C28" s="90" t="n">
-        <x:v>14</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D28" s="89" t="str">
         <x:v>Не BBx</x:v>
@@ -5588,47 +5584,61 @@
     </x:row>
     <x:row r="29" ht="27" customHeight="1">
       <x:c r="A29" s="89" t="str">
-        <x:v>[J-8]x dis</x:v>
+        <x:v>K/Qx con</x:v>
       </x:c>
       <x:c r="B29" s="89" t="str">
-        <x:v>Старшая J/T/9/8; lower gap &gt;1</x:v>
+        <x:v>Старшая K/Q; lower gap =1</x:v>
       </x:c>
       <x:c r="C29" s="90" t="n">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="D29" s="89" t="str"/>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D29" s="89" t="str">
+        <x:v>Не BBx</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="27" customHeight="1">
       <x:c r="A30" s="89" t="str">
-        <x:v>[J-8]x con</x:v>
+        <x:v>[J-8]x dis</x:v>
       </x:c>
       <x:c r="B30" s="89" t="str">
-        <x:v>Старшая J/T/9/8; lower gap =1</x:v>
+        <x:v>Старшая J/T/9/8; lower gap &gt;1</x:v>
       </x:c>
       <x:c r="C30" s="90" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D30" s="89" t="str">
-        <x:v>Включает JT9</x:v>
-      </x:c>
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="D30" s="89" t="str"/>
     </x:row>
     <x:row r="31" ht="27" customHeight="1">
       <x:c r="A31" s="89" t="str">
+        <x:v>[J-8]x con</x:v>
+      </x:c>
+      <x:c r="B31" s="89" t="str">
+        <x:v>Старшая J/T/9/8; lower gap =1</x:v>
+      </x:c>
+      <x:c r="C31" s="90" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="D31" s="89" t="str">
+        <x:v>Включает JT9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="27" customHeight="1">
+      <x:c r="A32" s="89" t="str">
         <x:v>[7-4]x</x:v>
       </x:c>
-      <x:c r="B31" s="89" t="str">
+      <x:c r="B32" s="89" t="str">
         <x:v>Старшая карта 7 или ниже</x:v>
       </x:c>
-      <x:c r="C31" s="90" t="n">
+      <x:c r="C32" s="90" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D31" s="89" t="str"/>
-    </x:row>
-    <x:row r="32" ht="27" customHeight="1">
-      <x:c r="A32" s="3"/>
-      <x:c r="B32" s="3"/>
-      <x:c r="C32" s="3"/>
-      <x:c r="D32" s="3"/>
+      <x:c r="D32" s="89" t="str"/>
+    </x:row>
+    <x:row r="33" ht="27" customHeight="1">
+      <x:c r="A33" s="3"/>
+      <x:c r="B33" s="3"/>
+      <x:c r="C33" s="3"/>
+      <x:c r="D33" s="3"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Place weak pairs after second pairs
</commit_message>
<xml_diff>
--- a/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_simplified_flop_strategy.xlsx
+++ b/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_simplified_flop_strategy.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R632a36dcb6814cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="Rda6ad3827c5b44be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="R5f43fc1e9cf7422c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="Rfdb2c4ae71734f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R753442d1c9fe477a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="R1ffd342a21e3471f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="Rb2fb9284317941f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="8" r:id="Re04fd1ba9ffd4e9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0b36e0fdd7714686"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="R133415c49bff4083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="R14c6ffeaba0a41fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="R9f6bd8fee2774d00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R488b630f13114caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="R4bc2df99ca164e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="R507a99126f4d4122"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="8" r:id="R5eecf4a51d1346fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1697,7 +1697,7 @@
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="37" t="str">
-        <x:v>Third pair</x:v>
+        <x:v>Weak pair</x:v>
       </x:c>
       <x:c r="B12" s="41" t="str">
         <x:v>X</x:v>
@@ -1726,14 +1726,14 @@
       <x:c r="J12" s="41" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="K12" s="61" t="str">
-        <x:v>X</x:v>
+      <x:c r="K12" s="62" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="L12" s="61" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="M12" s="61" t="str">
-        <x:v>X</x:v>
+      <x:c r="M12" s="62" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="N12" s="65" t="str">
         <x:v>X/D</x:v>
@@ -1741,7 +1741,7 @@
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="37" t="str">
-        <x:v>Weak pair</x:v>
+        <x:v>Third pair</x:v>
       </x:c>
       <x:c r="B13" s="41" t="str">
         <x:v>X</x:v>
@@ -1770,14 +1770,14 @@
       <x:c r="J13" s="41" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="K13" s="62" t="str">
-        <x:v>—</x:v>
+      <x:c r="K13" s="61" t="str">
+        <x:v>X</x:v>
       </x:c>
       <x:c r="L13" s="61" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="M13" s="62" t="str">
-        <x:v>—</x:v>
+      <x:c r="M13" s="61" t="str">
+        <x:v>X</x:v>
       </x:c>
       <x:c r="N13" s="65" t="str">
         <x:v>X/D</x:v>
@@ -2408,90 +2408,90 @@
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="37" t="str">
-        <x:v>Third pair</x:v>
+        <x:v>Weak pair</x:v>
       </x:c>
       <x:c r="B12" s="71" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C12" s="75" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="D12" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="E12" s="75" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="F12" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G12" s="75" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="H12" s="45" t="str">
+      <x:c r="C12" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="I12" s="75" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="J12" s="45" t="str">
+      <x:c r="D12" s="45" t="str">
+        <x:v>X/B</x:v>
+      </x:c>
+      <x:c r="E12" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="K12" s="61" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="L12" s="65" t="str">
+      <x:c r="F12" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G12" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="M12" s="61" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="N12" s="65" t="str">
-        <x:v>B/X</x:v>
+      <x:c r="H12" s="71" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="I12" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="J12" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="K12" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="L12" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="M12" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="N12" s="61" t="str">
+        <x:v>X</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="37" t="str">
-        <x:v>Weak pair</x:v>
+        <x:v>Third pair</x:v>
       </x:c>
       <x:c r="B13" s="71" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C13" s="65" t="str">
+      <x:c r="C13" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D13" s="71" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E13" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F13" s="71" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G13" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H13" s="45" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="D13" s="45" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="E13" s="65" t="str">
+      <x:c r="I13" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="J13" s="45" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="F13" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G13" s="65" t="str">
+      <x:c r="K13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="L13" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="H13" s="71" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="I13" s="61" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="J13" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="K13" s="62" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="L13" s="61" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="M13" s="62" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="N13" s="61" t="str">
-        <x:v>X</x:v>
+      <x:c r="M13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="N13" s="65" t="str">
+        <x:v>B/X</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
@@ -3119,43 +3119,43 @@
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="37" t="str">
-        <x:v>Third pair</x:v>
+        <x:v>Weak pair</x:v>
       </x:c>
       <x:c r="B12" s="45" t="str">
+        <x:v>R/F</x:v>
+      </x:c>
+      <x:c r="C12" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D12" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E12" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F12" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G12" s="65" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="C12" s="65" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="D12" s="45" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="E12" s="65" t="str">
+      <x:c r="H12" s="45" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="I12" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="J12" s="45" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="F12" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G12" s="61" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H12" s="45" t="str">
-        <x:v>C/F</x:v>
-      </x:c>
-      <x:c r="I12" s="65" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="J12" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K12" s="61" t="str">
-        <x:v>C</x:v>
+      <x:c r="K12" s="62" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="L12" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="M12" s="61" t="str">
-        <x:v>C</x:v>
+      <x:c r="M12" s="62" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="N12" s="61" t="str">
         <x:v>C</x:v>
@@ -3163,43 +3163,43 @@
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="37" t="str">
-        <x:v>Weak pair</x:v>
+        <x:v>Third pair</x:v>
       </x:c>
       <x:c r="B13" s="45" t="str">
-        <x:v>R/F</x:v>
-      </x:c>
-      <x:c r="C13" s="87" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D13" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E13" s="87" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F13" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G13" s="65" t="str">
         <x:v>C/F</x:v>
       </x:c>
+      <x:c r="C13" s="65" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="D13" s="45" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="E13" s="65" t="str">
+        <x:v>C/F</x:v>
+      </x:c>
+      <x:c r="F13" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
       <x:c r="H13" s="45" t="str">
+        <x:v>C/F</x:v>
+      </x:c>
+      <x:c r="I13" s="65" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="I13" s="87" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="J13" s="45" t="str">
-        <x:v>C/F</x:v>
-      </x:c>
-      <x:c r="K13" s="62" t="str">
-        <x:v>—</x:v>
+      <x:c r="J13" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K13" s="61" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="L13" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="M13" s="62" t="str">
-        <x:v>—</x:v>
+      <x:c r="M13" s="61" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="N13" s="61" t="str">
         <x:v>C</x:v>
@@ -3830,19 +3830,19 @@
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="37" t="str">
-        <x:v>Third pair</x:v>
-      </x:c>
-      <x:c r="B12" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C12" s="61" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="D12" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E12" s="61" t="str">
-        <x:v>C</x:v>
+        <x:v>Weak pair</x:v>
+      </x:c>
+      <x:c r="B12" s="45" t="str">
+        <x:v>C/F</x:v>
+      </x:c>
+      <x:c r="C12" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D12" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E12" s="65" t="str">
+        <x:v>F/C</x:v>
       </x:c>
       <x:c r="F12" s="41" t="str">
         <x:v>C</x:v>
@@ -3850,23 +3850,23 @@
       <x:c r="G12" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="H12" s="45" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="I12" s="61" t="str">
-        <x:v>C</x:v>
+      <x:c r="H12" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I12" s="87" t="str">
+        <x:v>F</x:v>
       </x:c>
       <x:c r="J12" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="K12" s="61" t="str">
-        <x:v>C</x:v>
+      <x:c r="K12" s="62" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="L12" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="M12" s="61" t="str">
-        <x:v>C</x:v>
+      <x:c r="M12" s="62" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="N12" s="61" t="str">
         <x:v>C</x:v>
@@ -3874,43 +3874,43 @@
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="37" t="str">
-        <x:v>Weak pair</x:v>
-      </x:c>
-      <x:c r="B13" s="45" t="str">
-        <x:v>C/F</x:v>
-      </x:c>
-      <x:c r="C13" s="87" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D13" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E13" s="65" t="str">
+        <x:v>Third pair</x:v>
+      </x:c>
+      <x:c r="B13" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D13" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F13" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H13" s="45" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="F13" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G13" s="61" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H13" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I13" s="87" t="str">
-        <x:v>F</x:v>
+      <x:c r="I13" s="61" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="J13" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="K13" s="62" t="str">
-        <x:v>—</x:v>
+      <x:c r="K13" s="61" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="L13" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="M13" s="62" t="str">
-        <x:v>—</x:v>
+      <x:c r="M13" s="61" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="N13" s="61" t="str">
         <x:v>C</x:v>
@@ -4541,43 +4541,43 @@
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="37" t="str">
-        <x:v>Third pair</x:v>
-      </x:c>
-      <x:c r="B12" s="45" t="str">
-        <x:v>R/F</x:v>
-      </x:c>
-      <x:c r="C12" s="86" t="str">
+        <x:v>Weak pair</x:v>
+      </x:c>
+      <x:c r="B12" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="D12" s="45" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-      <x:c r="E12" s="86" t="str">
+      <x:c r="C12" s="65" t="str">
+        <x:v>F/R</x:v>
+      </x:c>
+      <x:c r="D12" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E12" s="65" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="F12" s="45" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="G12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H12" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="F12" s="45" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-      <x:c r="G12" s="65" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-      <x:c r="H12" s="45" t="str">
-        <x:v>R/F</x:v>
-      </x:c>
       <x:c r="I12" s="65" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-      <x:c r="J12" s="45" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-      <x:c r="K12" s="65" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="L12" s="65" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="M12" s="61" t="str">
-        <x:v>C</x:v>
+        <x:v>C/F</x:v>
+      </x:c>
+      <x:c r="J12" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K12" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="L12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M12" s="62" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="N12" s="61" t="str">
         <x:v>C</x:v>
@@ -4585,43 +4585,43 @@
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="37" t="str">
-        <x:v>Weak pair</x:v>
-      </x:c>
-      <x:c r="B13" s="80" t="str">
+        <x:v>Third pair</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="str">
+        <x:v>R/F</x:v>
+      </x:c>
+      <x:c r="C13" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="C13" s="65" t="str">
-        <x:v>F/R</x:v>
-      </x:c>
-      <x:c r="D13" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E13" s="65" t="str">
-        <x:v>F/C</x:v>
+      <x:c r="D13" s="45" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+      <x:c r="E13" s="86" t="str">
+        <x:v>R</x:v>
       </x:c>
       <x:c r="F13" s="45" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+      <x:c r="G13" s="65" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+      <x:c r="H13" s="45" t="str">
+        <x:v>R/F</x:v>
+      </x:c>
+      <x:c r="I13" s="65" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+      <x:c r="J13" s="45" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+      <x:c r="K13" s="65" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="G13" s="61" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H13" s="80" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="I13" s="65" t="str">
-        <x:v>C/F</x:v>
-      </x:c>
-      <x:c r="J13" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K13" s="62" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="L13" s="61" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M13" s="62" t="str">
-        <x:v>—</x:v>
+      <x:c r="L13" s="65" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="M13" s="61" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="N13" s="61" t="str">
         <x:v>C</x:v>
@@ -5252,7 +5252,7 @@
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="37" t="str">
-        <x:v>Third pair</x:v>
+        <x:v>Weak pair</x:v>
       </x:c>
       <x:c r="B12" s="45" t="str">
         <x:v>F/C</x:v>
@@ -5272,23 +5272,23 @@
       <x:c r="G12" s="87" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="H12" s="45" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="I12" s="65" t="str">
-        <x:v>C/F</x:v>
-      </x:c>
-      <x:c r="J12" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="K12" s="61" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="L12" s="61" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="M12" s="61" t="str">
-        <x:v>C</x:v>
+      <x:c r="H12" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="J12" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="K12" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="L12" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="M12" s="62" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="N12" s="61" t="str">
         <x:v>C</x:v>
@@ -5296,7 +5296,7 @@
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="37" t="str">
-        <x:v>Weak pair</x:v>
+        <x:v>Third pair</x:v>
       </x:c>
       <x:c r="B13" s="45" t="str">
         <x:v>F/C</x:v>
@@ -5316,23 +5316,23 @@
       <x:c r="G13" s="87" t="str">
         <x:v>F</x:v>
       </x:c>
-      <x:c r="H13" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I13" s="61" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="J13" s="84" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="K13" s="62" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="L13" s="87" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="M13" s="62" t="str">
-        <x:v>—</x:v>
+      <x:c r="H13" s="45" t="str">
+        <x:v>F/C</x:v>
+      </x:c>
+      <x:c r="I13" s="65" t="str">
+        <x:v>C/F</x:v>
+      </x:c>
+      <x:c r="J13" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="L13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="M13" s="61" t="str">
+        <x:v>C</x:v>
       </x:c>
       <x:c r="N13" s="61" t="str">
         <x:v>C</x:v>

</xml_diff>